<commit_message>
updated files to have readable "sheet 2" and created subtracted peak list using a blank.
</commit_message>
<xml_diff>
--- a/forest_untargeted_results/forest4hr_blk2_qic.xlsx
+++ b/forest_untargeted_results/forest4hr_blk2_qic.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rawn54\Documents\github_projects\phytoncide_untargeted_targeted\forest_untargeted_results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E940954-B02D-4A38-9AB4-8FCD6ED22A8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3FD3B3B-800E-47C0-981C-7EC7C19B477B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="845" firstSheet="1" activeTab="2" autoFilterDateGrouping="0" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="845" firstSheet="1" activeTab="3" autoFilterDateGrouping="0" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="1" state="hidden" r:id="rId1"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1412" uniqueCount="293">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1393" uniqueCount="293">
   <si>
     <t>Sequence Overview</t>
   </si>
@@ -8699,418 +8699,442 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B99A71D8-31F4-4290-B18F-15342D094A5D}">
-  <dimension ref="A1:I82"/>
+  <dimension ref="A1:I79"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>57</v>
+        <v>58</v>
+      </c>
+      <c r="B1" t="s">
+        <v>59</v>
+      </c>
+      <c r="C1" t="s">
+        <v>60</v>
+      </c>
+      <c r="D1" t="s">
+        <v>61</v>
+      </c>
+      <c r="E1" t="s">
+        <v>62</v>
+      </c>
+      <c r="F1" t="s">
+        <v>63</v>
+      </c>
+      <c r="G1" t="s">
+        <v>64</v>
+      </c>
+      <c r="H1" t="s">
+        <v>65</v>
+      </c>
+      <c r="I1" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>58</v>
+      <c r="A2">
+        <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>59</v>
-      </c>
-      <c r="C2" t="s">
-        <v>60</v>
-      </c>
-      <c r="D2" t="s">
-        <v>61</v>
-      </c>
-      <c r="E2" t="s">
-        <v>62</v>
-      </c>
-      <c r="F2" t="s">
-        <v>63</v>
-      </c>
-      <c r="G2" t="s">
-        <v>64</v>
+        <v>72</v>
+      </c>
+      <c r="C2">
+        <v>3.4186333333333332</v>
+      </c>
+      <c r="D2">
+        <v>55.610783333333423</v>
+      </c>
+      <c r="E2">
+        <v>974</v>
+      </c>
+      <c r="F2">
+        <v>0.3488575832831553</v>
+      </c>
+      <c r="G2">
+        <v>0.15551296116369312</v>
       </c>
       <c r="H2" t="s">
-        <v>65</v>
+        <v>73</v>
       </c>
       <c r="I2" t="s">
-        <v>66</v>
+        <v>74</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>23</v>
+      <c r="A3">
+        <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>23</v>
-      </c>
-      <c r="C3" t="s">
-        <v>67</v>
-      </c>
-      <c r="D3" t="s">
-        <v>68</v>
-      </c>
-      <c r="E3" t="s">
-        <v>69</v>
-      </c>
-      <c r="F3" t="s">
-        <v>70</v>
-      </c>
-      <c r="G3" t="s">
-        <v>70</v>
+        <v>75</v>
+      </c>
+      <c r="C3">
+        <v>5.1581166666666665</v>
+      </c>
+      <c r="D3">
+        <v>8.9954000000000551</v>
+      </c>
+      <c r="E3">
+        <v>533</v>
+      </c>
+      <c r="F3">
+        <v>5.6429946074582835E-2</v>
+      </c>
+      <c r="G3">
+        <v>8.5101035215860807E-2</v>
       </c>
       <c r="H3" t="s">
-        <v>23</v>
+        <v>76</v>
       </c>
       <c r="I3" t="s">
-        <v>23</v>
+        <v>77</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>71</v>
+      <c r="A4">
+        <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>71</v>
-      </c>
-      <c r="C4" t="s">
-        <v>71</v>
-      </c>
-      <c r="D4" t="s">
-        <v>71</v>
-      </c>
-      <c r="E4" t="s">
-        <v>71</v>
-      </c>
-      <c r="F4" t="s">
-        <v>71</v>
-      </c>
-      <c r="G4" t="s">
-        <v>71</v>
+        <v>78</v>
+      </c>
+      <c r="C4">
+        <v>7.5727833333333336</v>
+      </c>
+      <c r="D4">
+        <v>218.09995833333406</v>
+      </c>
+      <c r="E4">
+        <v>4002</v>
+      </c>
+      <c r="F4">
+        <v>1.3681847263733384</v>
+      </c>
+      <c r="G4">
+        <v>0.63897625315924012</v>
       </c>
       <c r="H4" t="s">
-        <v>71</v>
+        <v>79</v>
       </c>
       <c r="I4" t="s">
-        <v>71</v>
+        <v>80</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A5">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>72</v>
+        <v>81</v>
       </c>
       <c r="C5">
-        <v>3.4186333333333332</v>
+        <v>7.6414499999999999</v>
       </c>
       <c r="D5">
-        <v>55.610783333333423</v>
+        <v>246.34030833333338</v>
       </c>
       <c r="E5">
-        <v>974</v>
+        <v>2888</v>
       </c>
       <c r="F5">
-        <v>0.3488575832831553</v>
+        <v>1.5453420987667057</v>
       </c>
       <c r="G5">
-        <v>0.15551296116369312</v>
+        <v>0.46111029963115574</v>
       </c>
       <c r="H5" t="s">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="I5" t="s">
-        <v>74</v>
+        <v>83</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A6">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>75</v>
+        <v>84</v>
       </c>
       <c r="C6">
-        <v>5.1581166666666665</v>
+        <v>7.7043833333333334</v>
       </c>
       <c r="D6">
-        <v>8.9954000000000551</v>
+        <v>3.248775000000049</v>
       </c>
       <c r="E6">
-        <v>533</v>
+        <v>206</v>
       </c>
       <c r="F6">
-        <v>5.6429946074582835E-2</v>
+        <v>2.0380216339290578E-2</v>
       </c>
       <c r="G6">
-        <v>8.5101035215860807E-2</v>
+        <v>3.2890831621889917E-2</v>
       </c>
       <c r="H6" t="s">
-        <v>76</v>
+        <v>23</v>
       </c>
       <c r="I6" t="s">
-        <v>77</v>
+        <v>85</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A7">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B7" t="s">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="C7">
-        <v>7.5727833333333336</v>
+        <v>7.7730500000000005</v>
       </c>
       <c r="D7">
-        <v>218.09995833333406</v>
+        <v>103.15405565912074</v>
       </c>
       <c r="E7">
-        <v>4002</v>
+        <v>1879.1105193075896</v>
       </c>
       <c r="F7">
-        <v>1.3681847263733384</v>
+        <v>0.64710605400745536</v>
       </c>
       <c r="G7">
-        <v>0.63897625315924012</v>
+        <v>0.30002673635664101</v>
       </c>
       <c r="H7" t="s">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="I7" t="s">
-        <v>80</v>
+        <v>88</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A8">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>81</v>
+        <v>89</v>
       </c>
       <c r="C8">
-        <v>7.6414499999999999</v>
+        <v>7.8646000000000003</v>
       </c>
       <c r="D8">
-        <v>246.34030833333338</v>
+        <v>115.50860833333418</v>
       </c>
       <c r="E8">
-        <v>2888</v>
+        <v>1942</v>
       </c>
       <c r="F8">
-        <v>1.5453420987667057</v>
+        <v>0.72460863768149464</v>
       </c>
       <c r="G8">
-        <v>0.46111029963115574</v>
+        <v>0.3100679369403409</v>
       </c>
       <c r="H8" t="s">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="I8" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A9">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="B9" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="C9">
-        <v>7.7043833333333334</v>
+        <v>8.5855666666666668</v>
       </c>
       <c r="D9">
-        <v>3.248775000000049</v>
+        <v>4.9652749999998491</v>
       </c>
       <c r="E9">
-        <v>206</v>
+        <v>333</v>
       </c>
       <c r="F9">
-        <v>2.0380216339290578E-2</v>
+        <v>3.1148164672550865E-2</v>
       </c>
       <c r="G9">
-        <v>3.2890831621889917E-2</v>
+        <v>5.3168188981016225E-2</v>
       </c>
       <c r="H9" t="s">
-        <v>23</v>
+        <v>92</v>
       </c>
       <c r="I9" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A10">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B10" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="C10">
-        <v>7.7730500000000005</v>
+        <v>9.729966666666666</v>
       </c>
       <c r="D10">
-        <v>103.15405565912074</v>
+        <v>64.316083333335527</v>
       </c>
       <c r="E10">
-        <v>1879.1105193075896</v>
+        <v>2277</v>
       </c>
       <c r="F10">
-        <v>0.64710605400745536</v>
+        <v>0.40346767394762623</v>
       </c>
       <c r="G10">
-        <v>0.30002673635664101</v>
+        <v>0.36355545438370557</v>
       </c>
       <c r="H10" t="s">
-        <v>87</v>
+        <v>23</v>
       </c>
       <c r="I10" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A11">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B11" t="s">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="C11">
-        <v>7.8646000000000003</v>
+        <v>9.8787333333333329</v>
       </c>
       <c r="D11">
-        <v>115.50860833333418</v>
+        <v>109.3940583333347</v>
       </c>
       <c r="E11">
-        <v>1942</v>
+        <v>3355</v>
       </c>
       <c r="F11">
-        <v>0.72460863768149464</v>
+        <v>0.68625084072190323</v>
       </c>
       <c r="G11">
-        <v>0.3100679369403409</v>
+        <v>0.53567349558951782</v>
       </c>
       <c r="H11" t="s">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="I11" t="s">
-        <v>85</v>
+        <v>98</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A12">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B12" t="s">
-        <v>91</v>
+        <v>99</v>
       </c>
       <c r="C12">
-        <v>8.5855666666666668</v>
+        <v>10.433766666666667</v>
       </c>
       <c r="D12">
-        <v>4.9652749999998491</v>
+        <v>54.634333333332222</v>
       </c>
       <c r="E12">
-        <v>333</v>
+        <v>1953</v>
       </c>
       <c r="F12">
-        <v>3.1148164672550865E-2</v>
+        <v>0.3427321168397961</v>
       </c>
       <c r="G12">
-        <v>5.3168188981016225E-2</v>
+        <v>0.31182424348325732</v>
       </c>
       <c r="H12" t="s">
-        <v>92</v>
+        <v>100</v>
       </c>
       <c r="I12" t="s">
-        <v>93</v>
+        <v>101</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A13">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B13" t="s">
-        <v>94</v>
+        <v>102</v>
       </c>
       <c r="C13">
-        <v>9.729966666666666</v>
+        <v>10.754200000000001</v>
       </c>
       <c r="D13">
-        <v>64.316083333335527</v>
+        <v>22.583125000000262</v>
       </c>
       <c r="E13">
-        <v>2277</v>
+        <v>1208</v>
       </c>
       <c r="F13">
-        <v>0.40346767394762623</v>
+        <v>0.14166846676585482</v>
       </c>
       <c r="G13">
-        <v>0.36355545438370557</v>
+        <v>0.19287439125846126</v>
       </c>
       <c r="H13" t="s">
-        <v>23</v>
+        <v>103</v>
       </c>
       <c r="I13" t="s">
-        <v>95</v>
+        <v>104</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A14">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B14" t="s">
-        <v>96</v>
+        <v>105</v>
       </c>
       <c r="C14">
-        <v>9.8787333333333329</v>
+        <v>10.811416666666666</v>
       </c>
       <c r="D14">
-        <v>109.3940583333347</v>
+        <v>8.9548000000003221</v>
       </c>
       <c r="E14">
-        <v>3355</v>
+        <v>375</v>
       </c>
       <c r="F14">
-        <v>0.68625084072190323</v>
+        <v>5.6175254141971387E-2</v>
       </c>
       <c r="G14">
-        <v>0.53567349558951782</v>
+        <v>5.9874086690333589E-2</v>
       </c>
       <c r="H14" t="s">
-        <v>97</v>
+        <v>106</v>
       </c>
       <c r="I14" t="s">
-        <v>98</v>
+        <v>107</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A15">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B15" t="s">
-        <v>99</v>
+        <v>108</v>
       </c>
       <c r="C15">
-        <v>10.433766666666667</v>
+        <v>11.051733333333333</v>
       </c>
       <c r="D15">
-        <v>54.634333333332222</v>
+        <v>168.95251666666616</v>
       </c>
       <c r="E15">
-        <v>1953</v>
+        <v>5339</v>
       </c>
       <c r="F15">
-        <v>0.3427321168397961</v>
+        <v>1.0598729800414624</v>
       </c>
       <c r="G15">
-        <v>0.31182424348325732</v>
+        <v>0.85244733023917607</v>
       </c>
       <c r="H15" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="I15" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.2">
@@ -9118,57 +9142,57 @@
         <v>4</v>
       </c>
       <c r="B16" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="C16">
-        <v>10.754200000000001</v>
+        <v>11.3264</v>
       </c>
       <c r="D16">
-        <v>22.583125000000262</v>
+        <v>14.043408333333705</v>
       </c>
       <c r="E16">
-        <v>1208</v>
+        <v>525</v>
       </c>
       <c r="F16">
-        <v>0.14166846676585482</v>
+        <v>8.8097113519505887E-2</v>
       </c>
       <c r="G16">
-        <v>0.19287439125846126</v>
+        <v>8.3823721366467027E-2</v>
       </c>
       <c r="H16" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="I16" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A17">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B17" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="C17">
-        <v>10.811416666666666</v>
+        <v>11.389333333333333</v>
       </c>
       <c r="D17">
-        <v>8.9548000000003221</v>
+        <v>2.0995249999999412</v>
       </c>
       <c r="E17">
-        <v>375</v>
+        <v>186</v>
       </c>
       <c r="F17">
-        <v>5.6175254141971387E-2</v>
+        <v>1.3170740882254761E-2</v>
       </c>
       <c r="G17">
-        <v>5.9874086690333589E-2</v>
+        <v>2.9697546998405461E-2</v>
       </c>
       <c r="H17" t="s">
-        <v>106</v>
+        <v>23</v>
       </c>
       <c r="I17" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.2">
@@ -9176,260 +9200,260 @@
         <v>2</v>
       </c>
       <c r="B18" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="C18">
-        <v>11.051733333333333</v>
+        <v>11.698316666666667</v>
       </c>
       <c r="D18">
-        <v>168.95251666666616</v>
+        <v>289.52043333332807</v>
       </c>
       <c r="E18">
-        <v>5339</v>
+        <v>11030</v>
       </c>
       <c r="F18">
-        <v>1.0598729800414624</v>
+        <v>1.8162196723313535</v>
       </c>
       <c r="G18">
-        <v>0.85244733023917607</v>
+        <v>1.7610964698516787</v>
       </c>
       <c r="H18" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="I18" t="s">
-        <v>104</v>
+        <v>114</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A19">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="B19" t="s">
-        <v>105</v>
+        <v>115</v>
       </c>
       <c r="C19">
-        <v>11.3264</v>
+        <v>11.829933333333333</v>
       </c>
       <c r="D19">
-        <v>14.043408333333705</v>
+        <v>156.13099245287731</v>
       </c>
       <c r="E19">
-        <v>525</v>
+        <v>3009.2914890593897</v>
       </c>
       <c r="F19">
-        <v>8.8097113519505887E-2</v>
+        <v>0.97944099036028542</v>
       </c>
       <c r="G19">
-        <v>8.3823721366467027E-2</v>
+        <v>0.48047621197979984</v>
       </c>
       <c r="H19" t="s">
-        <v>106</v>
+        <v>116</v>
       </c>
       <c r="I19" t="s">
-        <v>107</v>
+        <v>117</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A20">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="B20" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="C20">
-        <v>11.389333333333333</v>
+        <v>11.8757</v>
       </c>
       <c r="D20">
-        <v>2.0995249999999412</v>
+        <v>376.47741588045153</v>
       </c>
       <c r="E20">
-        <v>186</v>
+        <v>9913.7042483660116</v>
       </c>
       <c r="F20">
-        <v>1.3170740882254761E-2</v>
+        <v>2.3617182422607157</v>
       </c>
       <c r="G20">
-        <v>2.9697546998405461E-2</v>
+        <v>1.5828639669039866</v>
       </c>
       <c r="H20" t="s">
-        <v>23</v>
+        <v>116</v>
       </c>
       <c r="I20" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A21">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="B21" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="C21">
-        <v>11.698316666666667</v>
+        <v>12.07025</v>
       </c>
       <c r="D21">
-        <v>289.52043333332807</v>
+        <v>4.0251499999999716</v>
       </c>
       <c r="E21">
-        <v>11030</v>
+        <v>167.49999999999989</v>
       </c>
       <c r="F21">
-        <v>1.8162196723313535</v>
+        <v>2.5250572230484922E-2</v>
       </c>
       <c r="G21">
-        <v>1.7610964698516787</v>
+        <v>2.6743758721682317E-2</v>
       </c>
       <c r="H21" t="s">
-        <v>113</v>
+        <v>23</v>
       </c>
       <c r="I21" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A22">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="B22" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="C22">
-        <v>11.829933333333333</v>
+        <v>12.110300000000001</v>
       </c>
       <c r="D22">
-        <v>156.13099245287731</v>
+        <v>0.6232499999999721</v>
       </c>
       <c r="E22">
-        <v>3009.2914890593897</v>
+        <v>83.933980582522082</v>
       </c>
       <c r="F22">
-        <v>0.97944099036028542</v>
+        <v>3.9097720936236251E-3</v>
       </c>
       <c r="G22">
-        <v>0.48047621197979984</v>
+        <v>1.3401254479100544E-2</v>
       </c>
       <c r="H22" t="s">
-        <v>116</v>
+        <v>23</v>
       </c>
       <c r="I22" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A23">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B23" t="s">
-        <v>115</v>
+        <v>122</v>
       </c>
       <c r="C23">
-        <v>11.8757</v>
+        <v>12.178966666666668</v>
       </c>
       <c r="D23">
-        <v>376.47741588045153</v>
+        <v>13.604875000000355</v>
       </c>
       <c r="E23">
-        <v>9913.7042483660116</v>
+        <v>571.81779661016935</v>
       </c>
       <c r="F23">
-        <v>2.3617182422607157</v>
+        <v>8.5346106076600856E-2</v>
       </c>
       <c r="G23">
-        <v>1.5828639669039866</v>
+        <v>9.1298848867500851E-2</v>
       </c>
       <c r="H23" t="s">
-        <v>116</v>
+        <v>23</v>
       </c>
       <c r="I23" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A24">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B24" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="C24">
-        <v>12.07025</v>
+        <v>12.384966666666667</v>
       </c>
       <c r="D24">
-        <v>4.0251499999999716</v>
+        <v>8.9816916666664177</v>
       </c>
       <c r="E24">
-        <v>167.49999999999989</v>
+        <v>369</v>
       </c>
       <c r="F24">
-        <v>2.5250572230484922E-2</v>
+        <v>5.6343950953655519E-2</v>
       </c>
       <c r="G24">
-        <v>2.6743758721682317E-2</v>
+        <v>5.8916101303288254E-2</v>
       </c>
       <c r="H24" t="s">
         <v>23</v>
       </c>
       <c r="I24" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A25">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="B25" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="C25">
-        <v>12.110300000000001</v>
+        <v>12.596666666666668</v>
       </c>
       <c r="D25">
-        <v>0.6232499999999721</v>
+        <v>1.9451333333334269</v>
       </c>
       <c r="E25">
-        <v>83.933980582522082</v>
+        <v>176</v>
       </c>
       <c r="F25">
-        <v>3.9097720936236251E-3</v>
+        <v>1.2202211030957841E-2</v>
       </c>
       <c r="G25">
-        <v>1.3401254479100544E-2</v>
+        <v>2.8100904686663233E-2</v>
       </c>
       <c r="H25" t="s">
         <v>23</v>
       </c>
       <c r="I25" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A26">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="B26" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="C26">
-        <v>12.178966666666668</v>
+        <v>12.728283333333334</v>
       </c>
       <c r="D26">
-        <v>13.604875000000355</v>
+        <v>7.3588583333333695</v>
       </c>
       <c r="E26">
-        <v>571.81779661016935</v>
+        <v>342</v>
       </c>
       <c r="F26">
-        <v>8.5346106076600856E-2</v>
+        <v>4.6163592382828328E-2</v>
       </c>
       <c r="G26">
-        <v>9.1298848867500851E-2</v>
+        <v>5.4605167061584234E-2</v>
       </c>
       <c r="H26" t="s">
         <v>23</v>
       </c>
       <c r="I26" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.2">
@@ -9437,138 +9461,138 @@
         <v>4</v>
       </c>
       <c r="B27" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="C27">
-        <v>12.384966666666667</v>
+        <v>12.871333333333334</v>
       </c>
       <c r="D27">
-        <v>8.9816916666664177</v>
+        <v>0.89882499999999688</v>
       </c>
       <c r="E27">
-        <v>369</v>
+        <v>157</v>
       </c>
       <c r="F27">
-        <v>5.6343950953655519E-2</v>
+        <v>5.6385092692361012E-3</v>
       </c>
       <c r="G27">
-        <v>5.8916101303288254E-2</v>
+        <v>2.5067284294352996E-2</v>
       </c>
       <c r="H27" t="s">
         <v>23</v>
       </c>
       <c r="I27" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A28">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="B28" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="C28">
-        <v>12.596666666666668</v>
+        <v>12.9686</v>
       </c>
       <c r="D28">
-        <v>1.9451333333334269</v>
+        <v>2.1509333333332705</v>
       </c>
       <c r="E28">
-        <v>176</v>
+        <v>200</v>
       </c>
       <c r="F28">
-        <v>1.2202211030957841E-2</v>
+        <v>1.3493235654892324E-2</v>
       </c>
       <c r="G28">
-        <v>2.8100904686663233E-2</v>
+        <v>3.1932846234844582E-2</v>
       </c>
       <c r="H28" t="s">
         <v>23</v>
       </c>
       <c r="I28" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A29">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="B29" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="C29">
-        <v>12.728283333333334</v>
+        <v>13.483583333333334</v>
       </c>
       <c r="D29">
-        <v>7.3588583333333695</v>
+        <v>4.8187583333332604</v>
       </c>
       <c r="E29">
-        <v>342</v>
+        <v>257</v>
       </c>
       <c r="F29">
-        <v>4.6163592382828328E-2</v>
+        <v>3.0229036273699987E-2</v>
       </c>
       <c r="G29">
-        <v>5.4605167061584234E-2</v>
+        <v>4.1033707411775283E-2</v>
       </c>
       <c r="H29" t="s">
-        <v>23</v>
+        <v>135</v>
       </c>
       <c r="I29" t="s">
-        <v>129</v>
+        <v>136</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A30">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B30" t="s">
-        <v>130</v>
+        <v>137</v>
       </c>
       <c r="C30">
-        <v>12.871333333333334</v>
+        <v>13.91845</v>
       </c>
       <c r="D30">
-        <v>0.89882499999999688</v>
+        <v>0</v>
       </c>
       <c r="E30">
-        <v>157</v>
+        <v>0</v>
       </c>
       <c r="F30">
-        <v>5.6385092692361012E-3</v>
+        <v>0</v>
       </c>
       <c r="G30">
-        <v>2.5067284294352996E-2</v>
+        <v>0</v>
       </c>
       <c r="H30" t="s">
         <v>23</v>
       </c>
       <c r="I30" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A31">
-        <v>16</v>
+        <v>3</v>
       </c>
       <c r="B31" t="s">
         <v>132</v>
       </c>
       <c r="C31">
-        <v>12.9686</v>
+        <v>14.107266666666668</v>
       </c>
       <c r="D31">
-        <v>2.1509333333332705</v>
+        <v>3.7026916666667553</v>
       </c>
       <c r="E31">
-        <v>200</v>
+        <v>331</v>
       </c>
       <c r="F31">
-        <v>1.3493235654892324E-2</v>
+        <v>2.3227726513641522E-2</v>
       </c>
       <c r="G31">
-        <v>3.1932846234844582E-2</v>
+        <v>5.284886051866778E-2</v>
       </c>
       <c r="H31" t="s">
         <v>23</v>
@@ -9579,54 +9603,54 @@
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A32">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="B32" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="C32">
-        <v>13.483583333333334</v>
+        <v>14.170216666666667</v>
       </c>
       <c r="D32">
-        <v>4.8187583333332604</v>
+        <v>0.7607083333333069</v>
       </c>
       <c r="E32">
-        <v>257</v>
+        <v>94.670873786407924</v>
       </c>
       <c r="F32">
-        <v>3.0229036273699987E-2</v>
+        <v>4.7720757529941997E-3</v>
       </c>
       <c r="G32">
-        <v>4.1033707411775283E-2</v>
+        <v>1.5115552277698714E-2</v>
       </c>
       <c r="H32" t="s">
-        <v>135</v>
+        <v>23</v>
       </c>
       <c r="I32" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A33">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B33" t="s">
         <v>137</v>
       </c>
       <c r="C33">
-        <v>13.91845</v>
+        <v>14.771016666666666</v>
       </c>
       <c r="D33">
-        <v>0</v>
+        <v>0.93317499999999676</v>
       </c>
       <c r="E33">
-        <v>0</v>
+        <v>163</v>
       </c>
       <c r="F33">
-        <v>0</v>
+        <v>5.8539936999075452E-3</v>
       </c>
       <c r="G33">
-        <v>0</v>
+        <v>2.6025269681398334E-2</v>
       </c>
       <c r="H33" t="s">
         <v>23</v>
@@ -9640,312 +9664,312 @@
         <v>3</v>
       </c>
       <c r="B34" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="C34">
-        <v>14.107266666666668</v>
+        <v>14.85685</v>
       </c>
       <c r="D34">
-        <v>3.7026916666667553</v>
+        <v>0.85750000000008875</v>
       </c>
       <c r="E34">
-        <v>331</v>
+        <v>150</v>
       </c>
       <c r="F34">
-        <v>2.3227726513641522E-2</v>
+        <v>5.3792692663983243E-3</v>
       </c>
       <c r="G34">
-        <v>5.284886051866778E-2</v>
+        <v>2.3949634676133435E-2</v>
       </c>
       <c r="H34" t="s">
         <v>23</v>
       </c>
       <c r="I34" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A35">
-        <v>23</v>
+        <v>5</v>
       </c>
       <c r="B35" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="C35">
-        <v>14.170216666666667</v>
+        <v>15.097166666666666</v>
       </c>
       <c r="D35">
-        <v>0.7607083333333069</v>
+        <v>1.0648499999999963</v>
       </c>
       <c r="E35">
-        <v>94.670873786407924</v>
+        <v>186</v>
       </c>
       <c r="F35">
-        <v>4.7720757529941997E-3</v>
+        <v>6.6800173508147443E-3</v>
       </c>
       <c r="G35">
-        <v>1.5115552277698714E-2</v>
+        <v>2.9697546998405461E-2</v>
       </c>
       <c r="H35" t="s">
         <v>23</v>
       </c>
       <c r="I35" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A36">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="B36" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="C36">
-        <v>14.771016666666666</v>
+        <v>15.223050000000001</v>
       </c>
       <c r="D36">
-        <v>0.93317499999999676</v>
+        <v>4.4467703074434741</v>
       </c>
       <c r="E36">
-        <v>163</v>
+        <v>206.99999999999937</v>
       </c>
       <c r="F36">
-        <v>5.8539936999075452E-3</v>
+        <v>2.789548087412342E-2</v>
       </c>
       <c r="G36">
-        <v>2.6025269681398334E-2</v>
+        <v>3.3050495853064042E-2</v>
       </c>
       <c r="H36" t="s">
         <v>23</v>
       </c>
       <c r="I36" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A37">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B37" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="C37">
-        <v>14.85685</v>
+        <v>15.360383333333333</v>
       </c>
       <c r="D37">
-        <v>0.85750000000008875</v>
+        <v>1.0360333333334211</v>
       </c>
       <c r="E37">
-        <v>150</v>
+        <v>91.424708818635509</v>
       </c>
       <c r="F37">
-        <v>5.3792692663983243E-3</v>
+        <v>6.4992446285295699E-3</v>
       </c>
       <c r="G37">
-        <v>2.3949634676133435E-2</v>
+        <v>1.4597255843854637E-2</v>
       </c>
       <c r="H37" t="s">
         <v>23</v>
       </c>
       <c r="I37" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A38">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B38" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="C38">
-        <v>15.097166666666666</v>
+        <v>15.480550000000001</v>
       </c>
       <c r="D38">
-        <v>1.0648499999999963</v>
+        <v>5.4079833333334726</v>
       </c>
       <c r="E38">
-        <v>186</v>
+        <v>203.28963795255964</v>
       </c>
       <c r="F38">
-        <v>6.6800173508147443E-3</v>
+        <v>3.3925362726754643E-2</v>
       </c>
       <c r="G38">
-        <v>2.9697546998405461E-2</v>
+        <v>3.2458083749381562E-2</v>
       </c>
       <c r="H38" t="s">
         <v>23</v>
       </c>
       <c r="I38" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A39">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B39" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="C39">
-        <v>15.223050000000001</v>
+        <v>15.617866666666666</v>
       </c>
       <c r="D39">
-        <v>4.4467703074434741</v>
+        <v>7.8979250000000718</v>
       </c>
       <c r="E39">
-        <v>206.99999999999937</v>
+        <v>257.54646544876903</v>
       </c>
       <c r="F39">
-        <v>2.789548087412342E-2</v>
+        <v>4.9545265563632625E-2</v>
       </c>
       <c r="G39">
-        <v>3.3050495853064042E-2</v>
+        <v>4.1120958397516269E-2</v>
       </c>
       <c r="H39" t="s">
         <v>23</v>
       </c>
       <c r="I39" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A40">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="B40" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="C40">
-        <v>15.360383333333333</v>
+        <v>15.7037</v>
       </c>
       <c r="D40">
-        <v>1.0360333333334211</v>
+        <v>1.8020166666667601</v>
       </c>
       <c r="E40">
-        <v>91.424708818635509</v>
+        <v>163</v>
       </c>
       <c r="F40">
-        <v>6.4992446285295699E-3</v>
+        <v>1.1304411513162744E-2</v>
       </c>
       <c r="G40">
-        <v>1.4597255843854637E-2</v>
+        <v>2.6025269681398334E-2</v>
       </c>
       <c r="H40" t="s">
         <v>23</v>
       </c>
       <c r="I40" t="s">
-        <v>144</v>
+        <v>138</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A41">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B41" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="C41">
-        <v>15.480550000000001</v>
+        <v>15.921133333333334</v>
       </c>
       <c r="D41">
-        <v>5.4079833333334726</v>
+        <v>1.1850749999999959</v>
       </c>
       <c r="E41">
-        <v>203.28963795255964</v>
+        <v>207</v>
       </c>
       <c r="F41">
-        <v>3.3925362726754643E-2</v>
+        <v>7.4342128581647961E-3</v>
       </c>
       <c r="G41">
-        <v>3.2458083749381562E-2</v>
+        <v>3.3050495853064139E-2</v>
       </c>
       <c r="H41" t="s">
         <v>23</v>
       </c>
       <c r="I41" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A42">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="B42" t="s">
-        <v>145</v>
+        <v>137</v>
       </c>
       <c r="C42">
-        <v>15.617866666666666</v>
+        <v>16.006966666666667</v>
       </c>
       <c r="D42">
-        <v>7.8979250000000718</v>
+        <v>2.2996250000003204</v>
       </c>
       <c r="E42">
-        <v>257.54646544876903</v>
+        <v>219</v>
       </c>
       <c r="F42">
-        <v>4.9545265563632625E-2</v>
+        <v>1.4426008264421796E-2</v>
       </c>
       <c r="G42">
-        <v>4.1120958397516269E-2</v>
+        <v>3.4966466627154816E-2</v>
       </c>
       <c r="H42" t="s">
         <v>23</v>
       </c>
       <c r="I42" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A43">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B43" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="C43">
-        <v>15.7037</v>
+        <v>16.109966666666669</v>
       </c>
       <c r="D43">
-        <v>1.8020166666667601</v>
+        <v>4.7547416666666606</v>
       </c>
       <c r="E43">
-        <v>163</v>
+        <v>380.42571785268285</v>
       </c>
       <c r="F43">
-        <v>1.1304411513162744E-2</v>
+        <v>2.9827446900479147E-2</v>
       </c>
       <c r="G43">
-        <v>2.6025269681398334E-2</v>
+        <v>6.0740379759850457E-2</v>
       </c>
       <c r="H43" t="s">
         <v>23</v>
       </c>
       <c r="I43" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A44">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="B44" t="s">
         <v>137</v>
       </c>
       <c r="C44">
-        <v>15.921133333333334</v>
+        <v>16.190066666666667</v>
       </c>
       <c r="D44">
-        <v>1.1850749999999959</v>
+        <v>10.175791666666523</v>
       </c>
       <c r="E44">
-        <v>207</v>
+        <v>284</v>
       </c>
       <c r="F44">
-        <v>7.4342128581647961E-3</v>
+        <v>6.3834779444624776E-2</v>
       </c>
       <c r="G44">
-        <v>3.3050495853064139E-2</v>
+        <v>4.5344641653479303E-2</v>
       </c>
       <c r="H44" t="s">
         <v>23</v>
@@ -9962,19 +9986,19 @@
         <v>137</v>
       </c>
       <c r="C45">
-        <v>16.006966666666667</v>
+        <v>16.270183333333335</v>
       </c>
       <c r="D45">
-        <v>2.2996250000003204</v>
+        <v>2.9812999999999423</v>
       </c>
       <c r="E45">
-        <v>219</v>
+        <v>182</v>
       </c>
       <c r="F45">
-        <v>1.4426008264421796E-2</v>
+        <v>1.8702292086194002E-2</v>
       </c>
       <c r="G45">
-        <v>3.4966466627154816E-2</v>
+        <v>2.9058890073708567E-2</v>
       </c>
       <c r="H45" t="s">
         <v>23</v>
@@ -9985,141 +10009,141 @@
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A46">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B46" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="C46">
-        <v>16.109966666666669</v>
+        <v>16.356000000000002</v>
       </c>
       <c r="D46">
-        <v>4.7547416666666606</v>
+        <v>3.8457499999999385</v>
       </c>
       <c r="E46">
-        <v>380.42571785268285</v>
+        <v>183</v>
       </c>
       <c r="F46">
-        <v>2.9827446900479147E-2</v>
+        <v>2.4125160094750887E-2</v>
       </c>
       <c r="G46">
-        <v>6.0740379759850457E-2</v>
+        <v>2.921855430488279E-2</v>
       </c>
       <c r="H46" t="s">
         <v>23</v>
       </c>
       <c r="I46" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A47">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="B47" t="s">
-        <v>137</v>
+        <v>147</v>
       </c>
       <c r="C47">
-        <v>16.190066666666667</v>
+        <v>16.893866666666668</v>
       </c>
       <c r="D47">
-        <v>10.175791666666523</v>
+        <v>11.313074999999799</v>
       </c>
       <c r="E47">
-        <v>284</v>
+        <v>665.00000000000091</v>
       </c>
       <c r="F47">
-        <v>6.3834779444624776E-2</v>
+        <v>7.0969185604608562E-2</v>
       </c>
       <c r="G47">
-        <v>4.5344641653479303E-2</v>
+        <v>0.10617671373085837</v>
       </c>
       <c r="H47" t="s">
         <v>23</v>
       </c>
       <c r="I47" t="s">
-        <v>138</v>
+        <v>148</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A48">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B48" t="s">
-        <v>137</v>
+        <v>147</v>
       </c>
       <c r="C48">
-        <v>16.270183333333335</v>
+        <v>16.962533333333333</v>
       </c>
       <c r="D48">
-        <v>2.9812999999999423</v>
+        <v>13.005808333333249</v>
       </c>
       <c r="E48">
-        <v>182</v>
+        <v>705.44124312075223</v>
       </c>
       <c r="F48">
-        <v>1.8702292086194002E-2</v>
+        <v>8.1588040877153961E-2</v>
       </c>
       <c r="G48">
-        <v>2.9058890073708567E-2</v>
+        <v>0.11263373372146296</v>
       </c>
       <c r="H48" t="s">
         <v>23</v>
       </c>
       <c r="I48" t="s">
-        <v>138</v>
+        <v>148</v>
       </c>
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A49">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B49" t="s">
-        <v>137</v>
+        <v>147</v>
       </c>
       <c r="C49">
-        <v>16.356000000000002</v>
+        <v>17.117033333333335</v>
       </c>
       <c r="D49">
-        <v>3.8457499999999385</v>
+        <v>19.664458333333201</v>
       </c>
       <c r="E49">
-        <v>183</v>
+        <v>894.63778667638553</v>
       </c>
       <c r="F49">
-        <v>2.4125160094750887E-2</v>
+        <v>0.12335908612578281</v>
       </c>
       <c r="G49">
-        <v>2.921855430488279E-2</v>
+        <v>0.14284165438909355</v>
       </c>
       <c r="H49" t="s">
         <v>23</v>
       </c>
       <c r="I49" t="s">
-        <v>138</v>
+        <v>148</v>
       </c>
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A50">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B50" t="s">
         <v>147</v>
       </c>
       <c r="C50">
-        <v>16.893866666666668</v>
+        <v>17.174250000000001</v>
       </c>
       <c r="D50">
-        <v>11.313074999999799</v>
+        <v>20.361616666666777</v>
       </c>
       <c r="E50">
-        <v>665.00000000000091</v>
+        <v>615.37119406936972</v>
       </c>
       <c r="F50">
-        <v>7.0969185604608562E-2</v>
+        <v>0.12773249999903574</v>
       </c>
       <c r="G50">
-        <v>0.10617671373085837</v>
+        <v>9.825276858784944E-2</v>
       </c>
       <c r="H50" t="s">
         <v>23</v>
@@ -10136,19 +10160,19 @@
         <v>147</v>
       </c>
       <c r="C51">
-        <v>16.962533333333333</v>
+        <v>17.242916666666666</v>
       </c>
       <c r="D51">
-        <v>13.005808333333249</v>
+        <v>9.7395999999998253</v>
       </c>
       <c r="E51">
-        <v>705.44124312075223</v>
+        <v>515.41467676179127</v>
       </c>
       <c r="F51">
-        <v>8.1588040877153961E-2</v>
+        <v>6.1098461745780479E-2</v>
       </c>
       <c r="G51">
-        <v>0.11263373372146296</v>
+        <v>8.229328810108201E-2</v>
       </c>
       <c r="H51" t="s">
         <v>23</v>
@@ -10159,25 +10183,25 @@
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A52">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B52" t="s">
         <v>147</v>
       </c>
       <c r="C52">
-        <v>17.117033333333335</v>
+        <v>17.408850000000001</v>
       </c>
       <c r="D52">
-        <v>19.664458333333201</v>
+        <v>21.490299999999138</v>
       </c>
       <c r="E52">
-        <v>894.63778667638553</v>
+        <v>875.00776699028847</v>
       </c>
       <c r="F52">
-        <v>0.12335908612578281</v>
+        <v>0.13481295663634205</v>
       </c>
       <c r="G52">
-        <v>0.14284165438909355</v>
+        <v>0.139707442387978</v>
       </c>
       <c r="H52" t="s">
         <v>23</v>
@@ -10188,25 +10212,25 @@
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A53">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="B53" t="s">
         <v>147</v>
       </c>
       <c r="C53">
-        <v>17.174250000000001</v>
+        <v>17.477516666666666</v>
       </c>
       <c r="D53">
-        <v>20.361616666666777</v>
+        <v>16.460233333333065</v>
       </c>
       <c r="E53">
-        <v>615.37119406936972</v>
+        <v>864</v>
       </c>
       <c r="F53">
-        <v>0.12773249999903574</v>
+        <v>0.10325834086033195</v>
       </c>
       <c r="G53">
-        <v>9.825276858784944E-2</v>
+        <v>0.13794989573452859</v>
       </c>
       <c r="H53" t="s">
         <v>23</v>
@@ -10217,25 +10241,25 @@
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A54">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="B54" t="s">
         <v>147</v>
       </c>
       <c r="C54">
-        <v>17.242916666666666</v>
+        <v>17.546183333333335</v>
       </c>
       <c r="D54">
-        <v>9.7395999999998253</v>
+        <v>42.835949999999485</v>
       </c>
       <c r="E54">
-        <v>515.41467676179127</v>
+        <v>1340.906010060894</v>
       </c>
       <c r="F54">
-        <v>6.1098461745780479E-2</v>
+        <v>0.26871849484775356</v>
       </c>
       <c r="G54">
-        <v>8.229328810108201E-2</v>
+        <v>0.21409472717326741</v>
       </c>
       <c r="H54" t="s">
         <v>23</v>
@@ -10246,25 +10270,25 @@
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A55">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B55" t="s">
         <v>147</v>
       </c>
       <c r="C55">
-        <v>17.408850000000001</v>
+        <v>17.597666666666669</v>
       </c>
       <c r="D55">
-        <v>21.490299999999138</v>
+        <v>32.071658333333204</v>
       </c>
       <c r="E55">
-        <v>875.00776699028847</v>
+        <v>1024.0485594043344</v>
       </c>
       <c r="F55">
-        <v>0.13481295663634205</v>
+        <v>0.20119193702030222</v>
       </c>
       <c r="G55">
-        <v>0.139707442387978</v>
+        <v>0.16350392592236357</v>
       </c>
       <c r="H55" t="s">
         <v>23</v>
@@ -10275,25 +10299,25 @@
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A56">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="B56" t="s">
         <v>147</v>
       </c>
       <c r="C56">
-        <v>17.477516666666666</v>
+        <v>17.637733333333333</v>
       </c>
       <c r="D56">
-        <v>16.460233333333065</v>
+        <v>10.93991666666642</v>
       </c>
       <c r="E56">
-        <v>864</v>
+        <v>651.8217821782373</v>
       </c>
       <c r="F56">
-        <v>0.10325834086033195</v>
+        <v>6.8628288632013285E-2</v>
       </c>
       <c r="G56">
-        <v>0.13794989573452859</v>
+        <v>0.10407262371410006</v>
       </c>
       <c r="H56" t="s">
         <v>23</v>
@@ -10304,25 +10328,25 @@
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A57">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="B57" t="s">
         <v>147</v>
       </c>
       <c r="C57">
-        <v>17.546183333333335</v>
+        <v>17.820833333333333</v>
       </c>
       <c r="D57">
-        <v>42.835949999999485</v>
+        <v>3.4337583333332731</v>
       </c>
       <c r="E57">
-        <v>1340.906010060894</v>
+        <v>580.54271844665345</v>
       </c>
       <c r="F57">
-        <v>0.26871849484775356</v>
+        <v>2.1540653843424955E-2</v>
       </c>
       <c r="G57">
-        <v>0.21409472717326741</v>
+        <v>9.269190680457827E-2</v>
       </c>
       <c r="H57" t="s">
         <v>23</v>
@@ -10333,25 +10357,25 @@
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A58">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="B58" t="s">
         <v>147</v>
       </c>
       <c r="C58">
-        <v>17.597666666666669</v>
+        <v>17.912383333333334</v>
       </c>
       <c r="D58">
-        <v>32.071658333333204</v>
+        <v>30.974639206783337</v>
       </c>
       <c r="E58">
-        <v>1024.0485594043344</v>
+        <v>1210.2460167894405</v>
       </c>
       <c r="F58">
-        <v>0.20119193702030222</v>
+        <v>0.19431011629482092</v>
       </c>
       <c r="G58">
-        <v>0.16350392592236357</v>
+        <v>0.19323299980235167</v>
       </c>
       <c r="H58" t="s">
         <v>23</v>
@@ -10362,25 +10386,25 @@
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A59">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="B59" t="s">
         <v>147</v>
       </c>
       <c r="C59">
-        <v>17.637733333333333</v>
+        <v>18.015383333333332</v>
       </c>
       <c r="D59">
-        <v>10.93991666666642</v>
+        <v>1.0634500000001879</v>
       </c>
       <c r="E59">
-        <v>651.8217821782373</v>
+        <v>533.01914273823877</v>
       </c>
       <c r="F59">
-        <v>6.8628288632013285E-2</v>
+        <v>6.671234870381011E-3</v>
       </c>
       <c r="G59">
-        <v>0.10407262371410006</v>
+        <v>8.5104091626444264E-2</v>
       </c>
       <c r="H59" t="s">
         <v>23</v>
@@ -10391,25 +10415,25 @@
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A60">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B60" t="s">
         <v>147</v>
       </c>
       <c r="C60">
-        <v>17.820833333333333</v>
+        <v>18.055433333333333</v>
       </c>
       <c r="D60">
-        <v>3.4337583333332731</v>
+        <v>30.127658333332704</v>
       </c>
       <c r="E60">
-        <v>580.54271844665345</v>
+        <v>848.22832175666645</v>
       </c>
       <c r="F60">
-        <v>2.1540653843424955E-2</v>
+        <v>0.18899683561636058</v>
       </c>
       <c r="G60">
-        <v>9.269190680457827E-2</v>
+        <v>0.13543172285347951</v>
       </c>
       <c r="H60" t="s">
         <v>23</v>
@@ -10420,25 +10444,25 @@
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A61">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="B61" t="s">
         <v>147</v>
       </c>
       <c r="C61">
-        <v>17.912383333333334</v>
+        <v>18.106933333333334</v>
       </c>
       <c r="D61">
-        <v>30.974639206783337</v>
+        <v>30.463451856707536</v>
       </c>
       <c r="E61">
-        <v>1210.2460167894405</v>
+        <v>1063.9707295762328</v>
       </c>
       <c r="F61">
-        <v>0.19431011629482092</v>
+        <v>0.19110333565151585</v>
       </c>
       <c r="G61">
-        <v>0.19323299980235167</v>
+        <v>0.16987806852966625</v>
       </c>
       <c r="H61" t="s">
         <v>23</v>
@@ -10449,25 +10473,25 @@
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A62">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B62" t="s">
         <v>147</v>
       </c>
       <c r="C62">
-        <v>18.015383333333332</v>
+        <v>18.267150000000001</v>
       </c>
       <c r="D62">
-        <v>1.0634500000001879</v>
+        <v>11.276383333334479</v>
       </c>
       <c r="E62">
-        <v>533.01914273823877</v>
+        <v>811.9113607990048</v>
       </c>
       <c r="F62">
-        <v>6.671234870381011E-3</v>
+        <v>7.0739011429884757E-2</v>
       </c>
       <c r="G62">
-        <v>8.5104091626444264E-2</v>
+        <v>0.1296332032035902</v>
       </c>
       <c r="H62" t="s">
         <v>23</v>
@@ -10484,19 +10508,19 @@
         <v>147</v>
       </c>
       <c r="C63">
-        <v>18.055433333333333</v>
+        <v>18.330083333333334</v>
       </c>
       <c r="D63">
-        <v>30.127658333332704</v>
+        <v>12.755633333332895</v>
       </c>
       <c r="E63">
-        <v>848.22832175666645</v>
+        <v>1336.9126001456634</v>
       </c>
       <c r="F63">
-        <v>0.18899683561636058</v>
+        <v>8.0018642989430386E-2</v>
       </c>
       <c r="G63">
-        <v>0.13543172285347951</v>
+        <v>0.21345712244938861</v>
       </c>
       <c r="H63" t="s">
         <v>23</v>
@@ -10507,25 +10531,25 @@
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A64">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="B64" t="s">
         <v>147</v>
       </c>
       <c r="C64">
-        <v>18.106933333333334</v>
+        <v>18.404466666666668</v>
       </c>
       <c r="D64">
-        <v>30.463451856707536</v>
+        <v>30.543949999999597</v>
       </c>
       <c r="E64">
-        <v>1063.9707295762328</v>
+        <v>1162.3051711580501</v>
       </c>
       <c r="F64">
-        <v>0.19110333565151585</v>
+        <v>0.19160831662902381</v>
       </c>
       <c r="G64">
-        <v>0.16987806852966625</v>
+        <v>0.18557856154277363</v>
       </c>
       <c r="H64" t="s">
         <v>23</v>
@@ -10536,199 +10560,199 @@
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A65">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B65" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="C65">
-        <v>18.267150000000001</v>
+        <v>18.576133333333335</v>
       </c>
       <c r="D65">
-        <v>11.276383333334479</v>
+        <v>8.1295333333332351</v>
       </c>
       <c r="E65">
-        <v>811.9113607990048</v>
+        <v>265.00757134537002</v>
       </c>
       <c r="F65">
-        <v>7.0739011429884757E-2</v>
+        <v>5.0998191032251512E-2</v>
       </c>
       <c r="G65">
-        <v>0.1296332032035902</v>
+        <v>4.2312230134206527E-2</v>
       </c>
       <c r="H65" t="s">
-        <v>23</v>
+        <v>150</v>
       </c>
       <c r="I65" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A66">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B66" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="C66">
-        <v>18.330083333333334</v>
+        <v>18.702016666666665</v>
       </c>
       <c r="D66">
-        <v>12.755633333332895</v>
+        <v>8.2621083333332592</v>
       </c>
       <c r="E66">
-        <v>1336.9126001456634</v>
+        <v>324.91130526872996</v>
       </c>
       <c r="F66">
-        <v>8.0018642989430386E-2</v>
+        <v>5.1829860563438468E-2</v>
       </c>
       <c r="G66">
-        <v>0.21345712244938861</v>
+        <v>5.1876713755545006E-2</v>
       </c>
       <c r="H66" t="s">
-        <v>23</v>
+        <v>150</v>
       </c>
       <c r="I66" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A67">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="B67" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="C67">
-        <v>18.404466666666668</v>
+        <v>18.8279</v>
       </c>
       <c r="D67">
-        <v>30.543949999999597</v>
+        <v>10.319916666666181</v>
       </c>
       <c r="E67">
-        <v>1162.3051711580501</v>
+        <v>721.9814342919542</v>
       </c>
       <c r="F67">
-        <v>0.19160831662902381</v>
+        <v>6.4738904439397657E-2</v>
       </c>
       <c r="G67">
-        <v>0.18557856154277363</v>
+        <v>0.1152746106282876</v>
       </c>
       <c r="H67" t="s">
-        <v>23</v>
+        <v>150</v>
       </c>
       <c r="I67" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
     </row>
     <row r="68" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A68">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="B68" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="C68">
-        <v>18.576133333333335</v>
+        <v>18.930900000000001</v>
       </c>
       <c r="D68">
-        <v>8.1295333333332351</v>
+        <v>5.435350000000291</v>
       </c>
       <c r="E68">
-        <v>265.00757134537002</v>
+        <v>310.99417546414247</v>
       </c>
       <c r="F68">
-        <v>5.0998191032251512E-2</v>
+        <v>3.4097039308590871E-2</v>
       </c>
       <c r="G68">
-        <v>4.2312230134206527E-2</v>
+        <v>4.9654645925143681E-2</v>
       </c>
       <c r="H68" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="I68" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
     </row>
     <row r="69" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A69">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B69" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="C69">
-        <v>18.702016666666665</v>
+        <v>18.993833333333335</v>
       </c>
       <c r="D69">
-        <v>8.2621083333332592</v>
+        <v>1.5631999999998527</v>
       </c>
       <c r="E69">
-        <v>324.91130526872996</v>
+        <v>325.76110706481722</v>
       </c>
       <c r="F69">
-        <v>5.1829860563438468E-2</v>
+        <v>9.8062667256352161E-3</v>
       </c>
       <c r="G69">
-        <v>5.1876713755545006E-2</v>
+        <v>5.2012396705967759E-2</v>
       </c>
       <c r="H69" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="I69" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
     </row>
     <row r="70" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A70">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="B70" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="C70">
-        <v>18.8279</v>
+        <v>19.108283333333333</v>
       </c>
       <c r="D70">
-        <v>10.319916666666181</v>
+        <v>8.6984583333333276</v>
       </c>
       <c r="E70">
-        <v>721.9814342919542</v>
+        <v>365.46899708696901</v>
       </c>
       <c r="F70">
-        <v>6.4738904439397657E-2</v>
+        <v>5.4567171518998855E-2</v>
       </c>
       <c r="G70">
-        <v>0.1152746106282876</v>
+        <v>5.8352326437905222E-2</v>
       </c>
       <c r="H70" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="I70" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A71">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B71" t="s">
         <v>152</v>
       </c>
       <c r="C71">
-        <v>18.930900000000001</v>
+        <v>19.108283333333333</v>
       </c>
       <c r="D71">
-        <v>5.435350000000291</v>
+        <v>8.6984583333333276</v>
       </c>
       <c r="E71">
-        <v>310.99417546414247</v>
+        <v>365.46899708696901</v>
       </c>
       <c r="F71">
-        <v>3.4097039308590871E-2</v>
+        <v>5.4567171518998855E-2</v>
       </c>
       <c r="G71">
-        <v>4.9654645925143681E-2</v>
+        <v>5.8352326437905222E-2</v>
       </c>
       <c r="H71" t="s">
         <v>153</v>
@@ -10739,25 +10763,25 @@
     </row>
     <row r="72" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A72">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="B72" t="s">
         <v>152</v>
       </c>
       <c r="C72">
-        <v>18.993833333333335</v>
+        <v>19.279933333333332</v>
       </c>
       <c r="D72">
-        <v>1.5631999999998527</v>
+        <v>29.621066756961298</v>
       </c>
       <c r="E72">
-        <v>325.76110706481722</v>
+        <v>539.00419433764523</v>
       </c>
       <c r="F72">
-        <v>9.8062667256352161E-3</v>
+        <v>0.18581888518208572</v>
       </c>
       <c r="G72">
-        <v>5.2012396705967759E-2</v>
+        <v>8.6059690288601554E-2</v>
       </c>
       <c r="H72" t="s">
         <v>153</v>
@@ -10768,118 +10792,118 @@
     </row>
     <row r="73" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A73">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="B73" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="C73">
-        <v>19.108283333333333</v>
+        <v>19.377200000000002</v>
       </c>
       <c r="D73">
-        <v>8.6984583333333276</v>
+        <v>3.5158193465387093</v>
       </c>
       <c r="E73">
-        <v>365.46899708696901</v>
+        <v>305.21584619865894</v>
       </c>
       <c r="F73">
-        <v>5.4567171518998855E-2</v>
+        <v>2.2055439016959024E-2</v>
       </c>
       <c r="G73">
-        <v>5.8352326437905222E-2</v>
+        <v>4.8732053425498745E-2</v>
       </c>
       <c r="H73" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="I73" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
     </row>
     <row r="74" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A74">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B74" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="C74">
-        <v>19.108283333333333</v>
+        <v>19.428699999999999</v>
       </c>
       <c r="D74">
-        <v>8.6984583333333276</v>
+        <v>12.200358333333455</v>
       </c>
       <c r="E74">
-        <v>365.46899708696901</v>
+        <v>327.19438559322111</v>
       </c>
       <c r="F74">
-        <v>5.4567171518998855E-2</v>
+        <v>7.6535291686927742E-2</v>
       </c>
       <c r="G74">
-        <v>5.8352326437905222E-2</v>
+        <v>5.2241240020263882E-2</v>
       </c>
       <c r="H74" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="I74" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
     </row>
     <row r="75" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A75">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B75" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="C75">
-        <v>19.279933333333332</v>
+        <v>19.657583333333335</v>
       </c>
       <c r="D75">
-        <v>29.621066756961298</v>
+        <v>5.3853333333332927</v>
       </c>
       <c r="E75">
-        <v>539.00419433764523</v>
+        <v>245.25336730979552</v>
       </c>
       <c r="F75">
-        <v>0.18581888518208572</v>
+        <v>3.378327473971688E-2</v>
       </c>
       <c r="G75">
-        <v>8.6059690288601554E-2</v>
+        <v>3.9158190334407789E-2</v>
       </c>
       <c r="H75" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="I75" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
     </row>
     <row r="76" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A76">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B76" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="C76">
-        <v>19.377200000000002</v>
+        <v>19.766300000000001</v>
       </c>
       <c r="D76">
-        <v>3.5158193465387093</v>
+        <v>22.833633333332756</v>
       </c>
       <c r="E76">
-        <v>305.21584619865894</v>
+        <v>651.45762711864359</v>
       </c>
       <c r="F76">
-        <v>2.2055439016959024E-2</v>
+        <v>0.14323995572034112</v>
       </c>
       <c r="G76">
-        <v>4.8732053425498745E-2</v>
+        <v>0.10401448117648181</v>
       </c>
       <c r="H76" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="I76" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.2">
@@ -10890,19 +10914,19 @@
         <v>149</v>
       </c>
       <c r="C77">
-        <v>19.428699999999999</v>
+        <v>19.806350000000002</v>
       </c>
       <c r="D77">
-        <v>12.200358333333455</v>
+        <v>10.254724999999809</v>
       </c>
       <c r="E77">
-        <v>327.19438559322111</v>
+        <v>513.73200166458082</v>
       </c>
       <c r="F77">
-        <v>7.6535291686927742E-2</v>
+        <v>6.4329944055813201E-2</v>
       </c>
       <c r="G77">
-        <v>5.2241240020263882E-2</v>
+        <v>8.2024625075369895E-2</v>
       </c>
       <c r="H77" t="s">
         <v>150</v>
@@ -10913,25 +10937,25 @@
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A78">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B78" t="s">
         <v>149</v>
       </c>
       <c r="C78">
-        <v>19.657583333333335</v>
+        <v>19.886466666666667</v>
       </c>
       <c r="D78">
-        <v>5.3853333333332927</v>
+        <v>19.661258333333663</v>
       </c>
       <c r="E78">
-        <v>245.25336730979552</v>
+        <v>476.17815533980684</v>
       </c>
       <c r="F78">
-        <v>3.378327473971688E-2</v>
+        <v>0.12333901188479157</v>
       </c>
       <c r="G78">
-        <v>3.9158190334407789E-2</v>
+        <v>7.6028619074289941E-2</v>
       </c>
       <c r="H78" t="s">
         <v>150</v>
@@ -10941,106 +10965,19 @@
       </c>
     </row>
     <row r="79" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A79">
-        <v>7</v>
-      </c>
-      <c r="B79" t="s">
-        <v>152</v>
-      </c>
-      <c r="C79">
-        <v>19.766300000000001</v>
+      <c r="A79" t="s">
+        <v>155</v>
       </c>
       <c r="D79">
-        <v>22.833633333332756</v>
+        <v>2623.6900281335475</v>
       </c>
       <c r="E79">
-        <v>651.45762711864359</v>
+        <v>78991.129683628038</v>
       </c>
       <c r="F79">
-        <v>0.14323995572034112</v>
+        <v>16.458933099583774</v>
       </c>
       <c r="G79">
-        <v>0.10401448117648181</v>
-      </c>
-      <c r="H79" t="s">
-        <v>153</v>
-      </c>
-      <c r="I79" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="80" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A80">
-        <v>8</v>
-      </c>
-      <c r="B80" t="s">
-        <v>149</v>
-      </c>
-      <c r="C80">
-        <v>19.806350000000002</v>
-      </c>
-      <c r="D80">
-        <v>10.254724999999809</v>
-      </c>
-      <c r="E80">
-        <v>513.73200166458082</v>
-      </c>
-      <c r="F80">
-        <v>6.4329944055813201E-2</v>
-      </c>
-      <c r="G80">
-        <v>8.2024625075369895E-2</v>
-      </c>
-      <c r="H80" t="s">
-        <v>150</v>
-      </c>
-      <c r="I80" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="81" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A81">
-        <v>7</v>
-      </c>
-      <c r="B81" t="s">
-        <v>149</v>
-      </c>
-      <c r="C81">
-        <v>19.886466666666667</v>
-      </c>
-      <c r="D81">
-        <v>19.661258333333663</v>
-      </c>
-      <c r="E81">
-        <v>476.17815533980684</v>
-      </c>
-      <c r="F81">
-        <v>0.12333901188479157</v>
-      </c>
-      <c r="G81">
-        <v>7.6028619074289941E-2</v>
-      </c>
-      <c r="H81" t="s">
-        <v>150</v>
-      </c>
-      <c r="I81" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="82" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A82" t="s">
-        <v>155</v>
-      </c>
-      <c r="D82">
-        <v>2623.6900281335475</v>
-      </c>
-      <c r="E82">
-        <v>78991.129683628038</v>
-      </c>
-      <c r="F82">
-        <v>16.458933099583774</v>
-      </c>
-      <c r="G82">
         <v>0</v>
       </c>
     </row>

</xml_diff>